<commit_message>
Review of files for sprint 2
</commit_message>
<xml_diff>
--- a/docs/sprint2/task-board.xlsx
+++ b/docs/sprint2/task-board.xlsx
@@ -80,7 +80,7 @@
     <t xml:space="preserve">Марія (ТА)</t>
   </si>
   <si>
-    <t xml:space="preserve">Незалежний аудит SRS 1.0 (Розділ 3 F-10..140 та Розділ 4 GUI) — Аудит вимог</t>
+    <t xml:space="preserve">Незалежний аудит SRS 1.0 (Розділ 3 F-10..140, Розділ 4 GUI, Розділ 6 NF) — Аудит вимог</t>
   </si>
   <si>
     <t xml:space="preserve">ТА</t>
@@ -104,10 +104,10 @@
     <t xml:space="preserve">Незалежний аудит SRS 1.0 (Розділ 3 F-10..140 та Розділ 5 BL)</t>
   </si>
   <si>
-    <t xml:space="preserve">Аркуш аудиту КТ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Зведення дефектів SRS, модерація узгодження знахідок, заповнення requirements-defects.xlsx (27 дефектів)</t>
+    <t xml:space="preserve">Аркуш аудиту Дарії</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Зведення дефектів SRS, модерація узгодження знахідок, заповнення requirements-defects.xlsx</t>
   </si>
   <si>
     <t xml:space="preserve">ТА / КТ</t>
@@ -188,6 +188,7 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -208,12 +209,14 @@
       <sz val="10"/>
       <name val="Times New Roman"/>
       <family val="1"/>
+      <charset val="1"/>
     </font>
     <font>
       <b val="true"/>
       <sz val="10"/>
       <name val="Times New Roman"/>
       <family val="1"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -258,20 +261,24 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -488,7 +495,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="n">
         <v>2.2</v>
       </c>
@@ -750,12 +757,12 @@
       </c>
     </row>
     <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="3" t="s">
+      <c r="A13" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="B13" s="3"/>
-      <c r="C13" s="3"/>
-      <c r="D13" s="3"/>
+      <c r="B13" s="4"/>
+      <c r="C13" s="4"/>
+      <c r="D13" s="4"/>
       <c r="E13" s="3" t="s">
         <v>47</v>
       </c>
@@ -765,10 +772,10 @@
       <c r="G13" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="H13" s="3" t="s">
+      <c r="H13" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="I13" s="3"/>
+      <c r="I13" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>